<commit_message>
Align public release with CCL five-figure package
</commit_message>
<xml_diff>
--- a/Supplementary_Data_1.xlsx
+++ b/Supplementary_Data_1.xlsx
@@ -34,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
     </font>
   </fonts>
   <fills count="2">
@@ -72,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -80,6 +84,12 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -491,12 +501,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Descriptor dictionary</t>
+          <t>Declared descriptor dictionary</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Defines descriptor blocks, computation rules, interpretation boundaries, and caveats.</t>
+          <t>Defines BASE fields, generic descriptor types, and the single 78-variable AEM descriptor block.</t>
         </is>
       </c>
     </row>
@@ -542,12 +552,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Model benchmark metrics</t>
+          <t>Model-family benchmark metrics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fixed model-family checks under polymer-group CV with training-fold-only preprocessing and feature selection.</t>
+          <t>Eleven fixed tabular model-family checks under polymer-group validation.</t>
         </is>
       </c>
     </row>
@@ -559,12 +569,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Descriptor-family sensitivity and source-held-out offset-check metrics</t>
+          <t>Declared descriptor-block sensitivity and source offset-check metrics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Grouped descriptor-family sensitivity metrics, AEM-subset checks, and post hoc source-held-out offset-check R² values for the main AEM descriptors.</t>
+          <t>Compares BASE + GENERIC with the declared AEM descriptor block under grouped validation.</t>
         </is>
       </c>
     </row>
@@ -576,12 +586,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fixed-temperature stress-test metrics</t>
+          <t>Fixed-temperature checks for the declared AEM descriptor block</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Temperature-specific feature-set comparisons.</t>
+          <t>Tests the same two declared feature sets within four temperature slices.</t>
         </is>
       </c>
     </row>
@@ -593,12 +603,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Repeated polymer-holdout metrics</t>
+          <t>Repeated polymer-holdout AEM descriptor increment</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Uplift summary with interquartile range (IQR) and bootstrap confidence interval (CI) for mean ΔR².</t>
+          <t>Reports the repeated-holdout distribution for the declared AEM descriptor block.</t>
         </is>
       </c>
     </row>
@@ -610,12 +620,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aggregate source-heterogeneity categories</t>
+          <t>Aggregate source baseline-shift and exploratory polymer-theme diagnostics</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Aggregate source-held-out interpretation categories derived from source diagnostics and available method descriptions.</t>
+          <t>Provides aggregate evidence for the source-transfer interpretation</t>
         </is>
       </c>
     </row>
@@ -695,12 +705,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AEM response-selection summary</t>
+          <t>AEM response-profile selection</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Descriptor-level support, response amplitude, full-model importance, design axis, and main/SI placement.</t>
+          <t>Records support, amplitude, AEM-block importance, design axis, and literature basis for Fig. 3 and Fig. S6.</t>
         </is>
       </c>
     </row>
@@ -732,198 +742,296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Aggregate category</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Observed source-level pattern</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Plausible source of heterogeneity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Aggregate diagnostic</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Negative raw-R² group</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Remaining group</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Evidence basis</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Boundary of interpretation</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Reader note</t>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Interpretation boundary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>OH-exchange pretreatment and membrane conditioning</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Low-raw-R² source groups can show source-level residual shifts under source-held-out validation.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Alkaline medium, OH-exchange pretreatment, post-exchange handling before measurement, membrane conditioning, or measurement configuration.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Source diagnostics and available source-level method descriptions for low-raw-R² groups.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Aggregate interpretation only; study-specific experimental reanalysis is required before causal assignment.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Use as aggregate source-context interpretation.</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Source-context groups with defined raw R²</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>113 evaluable groups among 116 held-out groups; 3 singleton groups had undefined group-level R²</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Counts do not label article quality</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hydration and swelling state</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Several low-raw-R² groups report conductivity together with water uptake, swelling, or hydration-related measurements.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Hydration or swelling state and available water-uptake/swelling fields may shift the reported conductivity baseline.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Source diagnostics, extracted protocol notes, and available source-level method descriptions.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>The category motivates follow-up membrane characterization; it is not a model-derived morphology measurement.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Use as aggregate source-context interpretation.</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Median absolute mean shift (log10 units)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Raw held-out residual means</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Offset diagnostic, not calibrated performance</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Architecture-specific source behavior</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Some low-raw-R² groups cluster around block, comb, multication, fluorinated, side-chain, high-free-volume, or dense ionic-group architectures.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Architecture-dependent morphology, phase organization, cation placement, and transport-pathway differences are plausible contributors to source-level behavior not captured by pooled fitting.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Available source-level method descriptions and aggregate descriptor/source diagnostics.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>This is a plausible source-level interpretation, not evidence that the model establishes a transport law.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Use as aggregate source-context interpretation.</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Share with absolute mean shift &gt; 0.10</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Raw held-out residual means</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Descriptive aggregate</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Application and reporting setting</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Low-raw-R² groups include water-electrolysis-oriented and other electrochemical AEM reporting settings.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Different device motivation, test medium, reported protocol detail, and conductivity-measurement practice can change source transfer.</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Protocol metadata and source-held-out diagnostics.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>The category supports source-held-out checks, not prospective correction using held-out source information.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Use as aggregate source-context interpretation.</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Share retaining Spearman ρ ≥ 0.8</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>not used as contrast</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Within-source raw predictions</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Rank retention does not remove baseline shift</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Small source span or limited metadata</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>The most extreme negative R² values can occur in very small or narrow-span held-out source groups.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Small n, narrow target range, limited method details, or low-confidence source metadata can amplify source-level R² instability.</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Source-size, target-span, protocol-confidence, and method-description checks.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Extreme source-level R² values are interpreted with source size and target span; pooled raw source-held-out performance remains the prospective estimate.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Use as aggregate source-context interpretation.</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Exploratory title theme: rigid_aromatic_or_ether_free</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>27/34 (79.4%)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>49/79 (62.0%)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Rate difference +17.4%; OR 2.36; q=0.446</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Non-exclusive exploratory title category; no causal or article-quality assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Exploratory title theme: cyclic_or_heterocyclic_cation</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>20/34 (58.8%)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>36/79 (45.6%)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Rate difference +13.3%; OR 1.71; q=0.446</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Non-exclusive exploratory title category; no causal or article-quality assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Exploratory title theme: side_chain_or_spacer</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>13/34 (38.2%)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>24/79 (30.4%)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Rate difference +7.9%; OR 1.42; q=0.657</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Non-exclusive exploratory title category; no causal or article-quality assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Exploratory title theme: fluorinated_or_hydrophobic_balance</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2/34 (5.9%)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>1/79 (1.3%)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Rate difference +4.6%; OR 4.88; q=0.446</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Non-exclusive exploratory title category; no causal or article-quality assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Exploratory title theme: block_comb_or_segmented</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3/34 (8.8%)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>5/79 (6.3%)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Rate difference +2.5%; OR 1.43; q=0.695</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Non-exclusive exploratory title category; no causal or article-quality assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Exploratory title theme: dense_or_multication</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>3/34 (8.8%)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>11/79 (13.9%)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Rate difference -5.1%; OR 0.60; q=0.657</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Non-exclusive exploratory title category; no causal or article-quality assignment</t>
         </is>
       </c>
     </row>
@@ -981,7 +1089,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AEM conductivity/stability prediction [52]; AEM membrane ML [53]</t>
+          <t>AEM conductivity/stability prediction [24]; AEM membrane machine learning [25]</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1111,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Polymer informatics review [54]; materials informatics [55]; polymer informatics [56]; polyBERT [59]</t>
+          <t>Polymer and materials informatics [26–30]</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1133,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>data leakage [51]; copolymer informatics [60]</t>
+          <t>Data leakage [23]; copolymer informatics [30]</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1460,7 +1568,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Group definitions summarized; detailed mapping follows data-access conditions</t>
+          <t>Used as the primary grouped-validation key.</t>
         </is>
       </c>
     </row>
@@ -1492,19 +1600,19 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Group definitions summarized; detailed mapping follows data-access conditions</t>
+          <t>Used for the harder structural-transfer check.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Restricted source group</t>
+          <t>Source-context group</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Internal key representing literature reporting/source setting</t>
+          <t>Literature source and reporting context used as the source-held-out key</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1519,12 +1627,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>No calibration information used in preprocessing</t>
+          <t>Assigned before modeling; each held-out group is excluded from training</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Detailed source-group mapping and counts follow manuscript data-access conditions</t>
+          <t>Used for aggregate source-transfer diagnostics.</t>
         </is>
       </c>
     </row>
@@ -1556,39 +1664,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Public code provides schema; actual table restricted</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Internal extraction records/logs</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Manual extraction notes, source-group mapping, internal curation decision logs, and source identifiers</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Internal QA only</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Not part of public modeling table</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Follows manuscript data-access conditions</t>
+          <t>The public code package provides the released field schema.</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1997,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -1966,7 +2042,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2087,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2132,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2177,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2222,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2267,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2312,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2357,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2402,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Evaluation stratum from the stored aggregate predictions.</t>
+          <t>Descriptive subgroup check only; stratum size and composition differ, so values are not comparative evidence for missingness effects.</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2541,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>restricted source group</t>
+          <t>source-context group</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -2507,7 +2583,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Aggregate fold-size range only; per-context row counts and identifiers remain restricted.</t>
+          <t>All 116 source-context groups were held out in turn; group-level R² was defined for 113 groups, while three singleton groups contributed only to pooled metrics.</t>
         </is>
       </c>
     </row>
@@ -2568,12 +2644,12 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Full-model importance rank</t>
+          <t>AEM-block permutation-importance rank</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Full-model importance mean</t>
+          <t>AEM-block permutation-importance mean</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -2605,7 +2681,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Main Fig. 4</t>
+          <t>Main Fig. 3</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -2630,7 +2706,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Hydration, swelling control, ionic-domain connectivity, and block-domain transport are reported AEM conductivity axes [10,14].</t>
+          <t>Hydration, swelling control, and ionic-domain connectivity are established AEM conductivity axes [10,12,16].</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -2657,7 +2733,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Main Fig. 4</t>
+          <t>Main Fig. 3</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -2682,7 +2758,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Water-electrolysis-oriented high-free-volume polyelectrolytes and backbone/side-chain studies connect accessible volume, water channels, dimensional stability, and hydroxide conductivity [18,24,64].</t>
+          <t>High-free-volume and backbone/side-chain studies connect accessible volume, water organization, dimensional stability, and hydroxide conductivity [16,18,33].</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -2709,7 +2785,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Fig. S7</t>
+          <t>Fig. S6</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -2734,7 +2810,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Backbone structure and cation-tether placement affect morphology, swelling, and hydroxide conductivity [18,24].</t>
+          <t>Backbone structure and cation-tether placement affect morphology, swelling, and hydroxide conductivity [16,18,22].</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2761,7 +2837,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fig. S7</t>
+          <t>Fig. S6</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -2786,7 +2862,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Microphase separation, dense ionic groups, and connected hydrophilic domains affect hydroxide transport [10,14,39].</t>
+          <t>Microphase organization, dense ionic groups, and connected hydrophilic domains affect hydroxide transport [10,12,17].</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -2813,7 +2889,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Fig. S7</t>
+          <t>Fig. S6</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -2838,7 +2914,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Side-chain spacer architecture affects phase contrast, hydration, swelling, and conductivity [20,24].</t>
+          <t>Side-chain and spacer architecture affect phase contrast, hydration, swelling, and conductivity [18,21,22].</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2865,7 +2941,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fig. S7</t>
+          <t>Fig. S6</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -2890,7 +2966,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Backbone structure changes membrane morphology, hydration, and hydroxide conductivity [18].</t>
+          <t>Backbone structure changes membrane morphology, hydration, and hydroxide conductivity [16].</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2917,7 +2993,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fig. S7</t>
+          <t>Fig. S6</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -2942,7 +3018,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Hydration number, water uptake, and swelling jointly affect AEM conductivity [10,14,24].</t>
+          <t>Hydration, water uptake, and swelling jointly affect reported AEM conductivity [10,16,33].</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2969,7 +3045,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fig. S7</t>
+          <t>Fig. S6</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -2994,7 +3070,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Cation-spacer and side-chain placement studies link fixed-cation distance from the backbone to hydration, morphology, alkaline stability, and hydroxide conductivity [20,23,24].</t>
+          <t>Cation-spacer and side-chain placement studies link fixed-cation placement to hydration, morphology, alkaline stability, and hydroxide conductivity [18,21,22].</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -4024,7 +4100,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Formulation-level polymer identities used for polymer-group validation.</t>
+          <t>Polymer identity groups defined from curated structure, composition, and architecture information.</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4161,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Records without matched conductivity–temperature entries were not expanded before modeling.</t>
+          <t>Only matched conductivity-temperature observations were expanded into modeling rows.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4105,7 +4181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G130"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5374,7 +5450,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5411,7 +5487,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5448,7 +5524,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5485,7 +5561,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5522,7 +5598,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5559,7 +5635,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -5596,7 +5672,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5633,7 +5709,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5670,7 +5746,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5707,7 +5783,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5744,7 +5820,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5781,7 +5857,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5818,7 +5894,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5855,7 +5931,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5892,7 +5968,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5929,7 +6005,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5966,7 +6042,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -6003,7 +6079,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -6040,7 +6116,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -6077,7 +6153,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6114,7 +6190,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6151,7 +6227,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6188,7 +6264,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -6225,7 +6301,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -6262,7 +6338,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -6299,7 +6375,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -6336,7 +6412,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -6373,7 +6449,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -6410,7 +6486,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -6447,7 +6523,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -6484,7 +6560,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -6521,7 +6597,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -6558,7 +6634,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -6595,7 +6671,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -6632,7 +6708,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -6669,7 +6745,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6706,7 +6782,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6743,7 +6819,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -6780,7 +6856,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6817,7 +6893,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -6854,7 +6930,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6891,7 +6967,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6928,7 +7004,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6965,7 +7041,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -7002,7 +7078,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -7039,7 +7115,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -7076,7 +7152,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -7113,7 +7189,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -7150,7 +7226,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -7187,7 +7263,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -7224,7 +7300,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>AEM subset check</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -7261,7 +7337,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -7298,7 +7374,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -7335,7 +7411,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -7345,7 +7421,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7372,7 +7448,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -7382,7 +7458,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -7409,7 +7485,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -7419,7 +7495,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -7446,7 +7522,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7483,7 +7559,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -7493,7 +7569,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -7520,7 +7596,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -7530,7 +7606,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -7557,7 +7633,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -7594,7 +7670,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -7604,7 +7680,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>bottleneck-sensitive channel/hydration descriptor</t>
+          <t>bottleneck-sensitive transport/hydration descriptor</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -7631,7 +7707,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -7668,7 +7744,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -7705,7 +7781,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -7742,7 +7818,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -7779,7 +7855,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -7789,7 +7865,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>bottleneck-sensitive channel/hydration descriptor</t>
+          <t>bottleneck-sensitive transport/hydration descriptor</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -7816,7 +7892,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -7826,7 +7902,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -7853,7 +7929,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7890,7 +7966,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7927,7 +8003,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7937,7 +8013,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -7964,7 +8040,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -8001,7 +8077,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -8038,7 +8114,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -8048,7 +8124,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -8075,7 +8151,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -8112,7 +8188,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -8149,7 +8225,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -8159,7 +8235,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>microphase/channel balance descriptor</t>
+          <t>microphase/transport-organization descriptor</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8186,7 +8262,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -8223,7 +8299,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>AEM descriptors mixture/contrast</t>
+          <t>AEM descriptors</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -8233,7 +8309,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>bottleneck-sensitive channel/hydration descriptor</t>
+          <t>bottleneck-sensitive transport/hydration descriptor</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -8249,672 +8325,6 @@
       <c r="G112" t="inlineStr">
         <is>
           <t>Computed descriptor; not a direct experimental measurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>int__copoly_x_channel_harmonic</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>int__copoly_x_transport_heterogeneity</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_channel_formation</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_channel_index</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_charge_density</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_hydration_overlap</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_hydrophilic_density</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_transport_heterogeneity</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>int__iec_dev_x_water_network</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>int__invtemp_dev_x_cation_accessibility</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>int__invtemp_dev_x_channel_index</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>int__invtemp_dev_x_free_volume</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>int__invtemp_dev_x_hydration_overlap</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>int__invtemp_dev_x_transport_balance</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>int__invtemp_dev_x_water_network</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>int__thick_dev_x_channel_index</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>int__thick_dev_x_segregation</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>int__thick_dev_x_transport_balance</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>product of centered condition variable and AEM descriptor</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>extension-only; not default explanatory descriptor</t>
         </is>
       </c>
     </row>
@@ -9218,7 +8628,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>restricted source group</t>
+          <t>source-context group</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -9256,7 +8666,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Source-held-out offset check; source-level details follow the manuscript data-access route</t>
+          <t>Source-transfer check</t>
         </is>
       </c>
     </row>
@@ -9417,7 +8827,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Selected input features per fold (mean)</t>
+          <t>Selected input features per outer fold (mean; common model-agnostic matrix)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -9432,7 +8842,7 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Main-figure role</t>
+          <t>Figure/table location</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -9483,7 +8893,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -9534,7 +8944,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -9585,7 +8995,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Supplementary GBDT comparison</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -9636,7 +9046,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -9687,7 +9097,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -9738,7 +9148,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -9789,7 +9199,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -9840,7 +9250,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -9891,7 +9301,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -9942,7 +9352,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -9993,7 +9403,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Fig. 7A</t>
+          <t>Fig. S4; Table S5</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -10013,7 +9423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="10" max="10"/>
@@ -10133,26 +9543,26 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM subset check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>2049</v>
       </c>
       <c r="E3" t="n">
-        <v>0.129</v>
+        <v>0.128</v>
       </c>
       <c r="F3" t="n">
         <v>0.096</v>
       </c>
       <c r="G3" t="n">
-        <v>0.801</v>
+        <v>0.805</v>
       </c>
       <c r="H3" t="n">
-        <v>0.883</v>
+        <v>0.885</v>
       </c>
       <c r="I3" t="n">
-        <v>245.2</v>
+        <v>253.2</v>
       </c>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
@@ -10160,7 +9570,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Polymer-group CV</t>
+          <t>Chemistry-family CV</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -10170,26 +9580,26 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
+          <t>BASE + GENERIC</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>2049</v>
       </c>
       <c r="E4" t="n">
-        <v>0.128</v>
+        <v>0.158</v>
       </c>
       <c r="F4" t="n">
-        <v>0.096</v>
+        <v>0.12</v>
       </c>
       <c r="G4" t="n">
-        <v>0.805</v>
+        <v>0.702</v>
       </c>
       <c r="H4" t="n">
-        <v>0.885</v>
+        <v>0.841</v>
       </c>
       <c r="I4" t="n">
-        <v>253.2</v>
+        <v>238</v>
       </c>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
@@ -10197,7 +9607,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Polymer-group CV</t>
+          <t>Chemistry-family CV</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -10207,26 +9617,26 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>condition-descriptor interaction check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>2049</v>
       </c>
       <c r="E5" t="n">
-        <v>0.129</v>
+        <v>0.157</v>
       </c>
       <c r="F5" t="n">
-        <v>0.096</v>
+        <v>0.119</v>
       </c>
       <c r="G5" t="n">
-        <v>0.802</v>
+        <v>0.707</v>
       </c>
       <c r="H5" t="n">
-        <v>0.883</v>
+        <v>0.841</v>
       </c>
       <c r="I5" t="n">
-        <v>257.2</v>
+        <v>255</v>
       </c>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
@@ -10234,7 +9644,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chemistry-family CV</t>
+          <t>Source-held-out CV</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -10251,16 +9661,16 @@
         <v>2049</v>
       </c>
       <c r="E6" t="n">
-        <v>0.158</v>
+        <v>0.165</v>
       </c>
       <c r="F6" t="n">
-        <v>0.12</v>
+        <v>0.128</v>
       </c>
       <c r="G6" t="n">
-        <v>0.702</v>
+        <v>0.675</v>
       </c>
       <c r="H6" t="n">
-        <v>0.841</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="I6" t="n">
         <v>238</v>
@@ -10271,7 +9681,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Chemistry-family CV</t>
+          <t>Source-held-out CV</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -10281,260 +9691,38 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM subset check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>2049</v>
       </c>
       <c r="E7" t="n">
-        <v>0.16</v>
+        <v>0.164</v>
       </c>
       <c r="F7" t="n">
-        <v>0.121</v>
+        <v>0.126</v>
       </c>
       <c r="G7" t="n">
-        <v>0.694</v>
+        <v>0.679</v>
       </c>
       <c r="H7" t="n">
-        <v>0.832</v>
+        <v>0.821</v>
       </c>
       <c r="I7" t="n">
-        <v>245</v>
-      </c>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Chemistry-family CV</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>2049</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.157</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.119</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.707</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.841</v>
-      </c>
-      <c r="I8" t="n">
-        <v>255</v>
-      </c>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Chemistry-family CV</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>2049</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.159</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.697</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.833</v>
-      </c>
-      <c r="I9" t="n">
-        <v>259</v>
-      </c>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Source-held-out CV</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>2049</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.165</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.675</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.8139999999999999</v>
-      </c>
-      <c r="I10" t="n">
-        <v>238</v>
-      </c>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Source-held-out CV</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM subset check</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2049</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.164</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.8139999999999999</v>
-      </c>
-      <c r="I11" t="n">
-        <v>245</v>
-      </c>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Source-held-out CV</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2049</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.164</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.679</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="I12" t="n">
         <v>251</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J7" s="2" t="n">
         <v>0.871</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>0.891</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Post hoc offset-size check; raw held-out predictions remain the prospective estimate.</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Source-held-out CV</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>2049</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.166</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-      <c r="I13" t="n">
-        <v>253</v>
-      </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10547,7 +9735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10653,7 +9841,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM subset check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -10666,16 +9854,16 @@
         <v>0.143</v>
       </c>
       <c r="G3" t="n">
-        <v>0.107</v>
+        <v>0.106</v>
       </c>
       <c r="H3" t="n">
-        <v>0.736</v>
+        <v>0.737</v>
       </c>
       <c r="I3" t="n">
-        <v>0.842</v>
+        <v>0.837</v>
       </c>
       <c r="J3" t="n">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4">
@@ -10691,29 +9879,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
+          <t>BASE + GENERIC</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E4" t="n">
-        <v>215</v>
+        <v>355</v>
       </c>
       <c r="F4" t="n">
-        <v>0.143</v>
+        <v>0.132</v>
       </c>
       <c r="G4" t="n">
-        <v>0.106</v>
+        <v>0.099</v>
       </c>
       <c r="H4" t="n">
-        <v>0.737</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.837</v>
+        <v>0.796</v>
       </c>
       <c r="J4" t="n">
-        <v>250</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5">
@@ -10729,29 +9917,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>condition-descriptor interaction check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E5" t="n">
-        <v>215</v>
+        <v>355</v>
       </c>
       <c r="F5" t="n">
-        <v>0.146</v>
+        <v>0.132</v>
       </c>
       <c r="G5" t="n">
-        <v>0.11</v>
+        <v>0.099</v>
       </c>
       <c r="H5" t="n">
-        <v>0.725</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>0.832</v>
+        <v>0.799</v>
       </c>
       <c r="J5" t="n">
-        <v>254</v>
+        <v>251.4</v>
       </c>
     </row>
     <row r="6">
@@ -10771,22 +9959,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E6" t="n">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="F6" t="n">
         <v>0.132</v>
       </c>
       <c r="G6" t="n">
-        <v>0.099</v>
+        <v>0.097</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.664</v>
       </c>
       <c r="I6" t="n">
-        <v>0.796</v>
+        <v>0.778</v>
       </c>
       <c r="J6" t="n">
         <v>236</v>
@@ -10805,29 +9993,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM subset check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E7" t="n">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="F7" t="n">
-        <v>0.132</v>
+        <v>0.13</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1</v>
+        <v>0.096</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.671</v>
       </c>
       <c r="I7" t="n">
-        <v>0.798</v>
+        <v>0.774</v>
       </c>
       <c r="J7" t="n">
-        <v>243.4</v>
+        <v>251.2</v>
       </c>
     </row>
     <row r="8">
@@ -10843,29 +10031,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
+          <t>BASE + GENERIC</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E8" t="n">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="F8" t="n">
-        <v>0.132</v>
+        <v>0.121</v>
       </c>
       <c r="G8" t="n">
-        <v>0.099</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.701</v>
       </c>
       <c r="I8" t="n">
-        <v>0.799</v>
+        <v>0.788</v>
       </c>
       <c r="J8" t="n">
-        <v>251.4</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9">
@@ -10881,333 +10069,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>condition-descriptor interaction check</t>
+          <t>BASE + GENERIC + AEM descriptors</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E9" t="n">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="F9" t="n">
-        <v>0.132</v>
+        <v>0.12</v>
       </c>
       <c r="G9" t="n">
-        <v>0.099</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.703</v>
       </c>
       <c r="I9" t="n">
-        <v>0.799</v>
+        <v>0.791</v>
       </c>
       <c r="J9" t="n">
-        <v>255.4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>60</v>
-      </c>
-      <c r="E10" t="n">
-        <v>371</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.664</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.778</v>
-      </c>
-      <c r="J10" t="n">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM subset check</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>60</v>
-      </c>
-      <c r="E11" t="n">
-        <v>371</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.129</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.678</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.779</v>
-      </c>
-      <c r="J11" t="n">
-        <v>243.2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>60</v>
-      </c>
-      <c r="E12" t="n">
-        <v>371</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.671</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.774</v>
-      </c>
-      <c r="J12" t="n">
-        <v>251.2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>60</v>
-      </c>
-      <c r="E13" t="n">
-        <v>371</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.129</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.776</v>
-      </c>
-      <c r="J13" t="n">
-        <v>255.2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>80</v>
-      </c>
-      <c r="E14" t="n">
-        <v>410</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.701</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.788</v>
-      </c>
-      <c r="J14" t="n">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM subset check</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>80</v>
-      </c>
-      <c r="E15" t="n">
-        <v>410</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.08799999999999999</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.702</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="J15" t="n">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM descriptors</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>80</v>
-      </c>
-      <c r="E16" t="n">
-        <v>410</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.703</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0.791</v>
-      </c>
-      <c r="J16" t="n">
         <v>252</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Polymer-group CV</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>CatBoost</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>80</v>
-      </c>
-      <c r="E17" t="n">
-        <v>410</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.119</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.709</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="J17" t="n">
-        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -11221,7 +10105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11274,111 +10158,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BASE + GENERIC + AEM subset check vs BASE + GENERIC</t>
+          <t>BASE + GENERIC + AEM descriptors vs BASE + GENERIC</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.001</v>
+        <v>0.005</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-0.009 to +0.005</t>
+          <t>+0.000 to +0.010</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-0.007 to +0.005</t>
+          <t>-0.001 to +0.010</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.026</v>
+        <v>-0.023</v>
       </c>
       <c r="H2" t="n">
-        <v>0.023</v>
+        <v>0.032</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>effect size near zero; bootstrap CI crosses zero</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>BASE + GENERIC + AEM descriptors vs BASE + GENERIC</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>+0.000 to +0.010</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>-0.001 to +0.010</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>75</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-0.023</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
           <t>small positive median ΔR²; bootstrap CI crosses zero</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>condition-descriptor interaction check vs BASE + GENERIC</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-0.005 to +0.005</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>-0.004 to +0.008</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-0.028</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>effect size near zero; bootstrap CI crosses zero</t>
         </is>
       </c>
     </row>

</xml_diff>